<commit_message>
Atualiza aba 1.2 com fórmulas CORREL do Excel
Novas abas:
- Dados 1.2 - Matriz: Matriz de correlação completa
- Dados 1.2 - Pares: Tabela com pares e fórmulas =CORREL
- Dados 1.2 - Instruções: Como usar no Excel
</commit_message>
<xml_diff>
--- a/dados/Dados_Tratados_Exercicios.xlsx
+++ b/dados/Dados_Tratados_Exercicios.xlsx
@@ -9,16 +9,18 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados Originais" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.2" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.3" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.4" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.5" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.6" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.7" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.8" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.9" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.9 - Variância" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados Tratados" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.2 - Matriz" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.2 - Pares" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.2 - Instruções" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.3" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.4" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.5" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.6" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.7" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.8" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.9" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados 1.9 - Variância" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados Tratados" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -827,12 +829,12 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>PC1</t>
+          <t>EC_Casado</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>PC2</t>
+          <t>EC_Solteiro</t>
         </is>
       </c>
     </row>
@@ -852,11 +854,11 @@
       <c r="E2" t="n">
         <v>0</v>
       </c>
-      <c r="F2" t="n">
-        <v>-2.637417193953826</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.4346025964147514</v>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -875,11 +877,11 @@
       <c r="E3" t="n">
         <v>0</v>
       </c>
-      <c r="F3" t="n">
-        <v>-2.304957393348385</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.2811702192335956</v>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -898,11 +900,11 @@
       <c r="E4" t="n">
         <v>0</v>
       </c>
-      <c r="F4" t="n">
-        <v>-2.051605081387693</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.1530934413726104</v>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -921,11 +923,11 @@
       <c r="E5" t="n">
         <v>0</v>
       </c>
-      <c r="F5" t="n">
-        <v>-1.694292205197514</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.1122001138223545</v>
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -944,11 +946,11 @@
       <c r="E6" t="n">
         <v>0</v>
       </c>
-      <c r="F6" t="n">
-        <v>-1.388796700952167</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.008531624239318792</v>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -967,11 +969,11 @@
       <c r="E7" t="n">
         <v>0</v>
       </c>
-      <c r="F7" t="n">
-        <v>-0.9989894608366757</v>
-      </c>
-      <c r="G7" t="n">
-        <v>-0.05461118699078554</v>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -990,20 +992,18 @@
       <c r="E8" t="n">
         <v>0</v>
       </c>
-      <c r="F8" t="n">
-        <v>-0.6471666286186903</v>
-      </c>
-      <c r="G8" t="n">
-        <v>-0.08128390683026435</v>
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
         <v>49</v>
       </c>
-      <c r="B9" t="n">
-        <v>7500</v>
-      </c>
+      <c r="B9" t="inlineStr"/>
       <c r="C9" t="n">
         <v>1400</v>
       </c>
@@ -1013,11 +1013,11 @@
       <c r="E9" t="n">
         <v>1</v>
       </c>
-      <c r="F9" t="n">
-        <v>-0.4215809384164558</v>
-      </c>
-      <c r="G9" t="n">
-        <v>-0.2231836742363878</v>
+      <c r="F9" t="b">
+        <v>0</v>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1036,11 +1036,11 @@
       <c r="E10" t="n">
         <v>1</v>
       </c>
-      <c r="F10" t="n">
-        <v>0.08106134711526591</v>
-      </c>
-      <c r="G10" t="n">
-        <v>-0.1377036327012556</v>
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1059,11 +1059,11 @@
       <c r="E11" t="n">
         <v>1</v>
       </c>
-      <c r="F11" t="n">
-        <v>0.5512643247747445</v>
-      </c>
-      <c r="G11" t="n">
-        <v>-0.1839543170640381</v>
+      <c r="F11" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1082,11 +1082,11 @@
       <c r="E12" t="n">
         <v>1</v>
       </c>
-      <c r="F12" t="n">
-        <v>1.107503768669124</v>
-      </c>
-      <c r="G12" t="n">
-        <v>-0.08721285761735803</v>
+      <c r="F12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G12" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -1105,20 +1105,18 @@
       <c r="E13" t="n">
         <v>1</v>
       </c>
-      <c r="F13" t="n">
-        <v>1.597561315459733</v>
-      </c>
-      <c r="G13" t="n">
-        <v>-0.1004653549471876</v>
+      <c r="F13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
         <v>64</v>
       </c>
-      <c r="B14" t="n">
-        <v>7500</v>
-      </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
         <v>3200</v>
       </c>
@@ -1128,11 +1126,11 @@
       <c r="E14" t="n">
         <v>1</v>
       </c>
-      <c r="F14" t="n">
-        <v>1.451621009374509</v>
-      </c>
-      <c r="G14" t="n">
-        <v>-1.09292608982185</v>
+      <c r="F14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -1151,11 +1149,11 @@
       <c r="E15" t="n">
         <v>1</v>
       </c>
-      <c r="F15" t="n">
-        <v>2.97875949252056</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0.1345091924002882</v>
+      <c r="F15" t="b">
+        <v>1</v>
+      </c>
+      <c r="G15" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -1174,11 +1172,11 @@
       <c r="E16" t="n">
         <v>1</v>
       </c>
-      <c r="F16" t="n">
-        <v>4.377034344797472</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0.8372338327262088</v>
+      <c r="F16" t="b">
+        <v>1</v>
+      </c>
+      <c r="G16" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1192,76 +1190,135 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Componente</t>
+          <t>Variável</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Variância_%</t>
+          <t>Média_Classe_0</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Acumulada_%</t>
+          <t>Média_Classe_1</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>F_Statistic</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>P_Value</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Significativo</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PC1</t>
+          <t>Idade</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>95.17</v>
+        <v>34.57</v>
       </c>
       <c r="C2" t="n">
-        <v>95.17</v>
+        <v>59.88</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.6118</v>
+      </c>
+      <c r="E2" t="n">
+        <v>4.7e-05</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PC2</t>
+          <t>Renda_Mensal</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3.91</v>
+        <v>4500</v>
       </c>
       <c r="C3" t="n">
-        <v>99.08</v>
+        <v>14412.5</v>
+      </c>
+      <c r="D3" t="n">
+        <v>10.8889</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.00575</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PC3</t>
+          <t>Valor_Compras</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.89</v>
+        <v>738.5700000000001</v>
       </c>
       <c r="C4" t="n">
-        <v>99.95999999999999</v>
+        <v>2762.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>23.3116</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.00033</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>Numero_Compras</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.04</v>
+        <v>5.29</v>
       </c>
       <c r="C5" t="n">
-        <v>100</v>
+        <v>18</v>
+      </c>
+      <c r="D5" t="n">
+        <v>22.8448</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.00036</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1270,6 +1327,485 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Idade</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Renda_Mensal</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Valor_Compras</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Numero_Compras</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Classe</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>PC1</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>PC2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B2" t="n">
+        <v>2200</v>
+      </c>
+      <c r="C2" t="n">
+        <v>300</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-2.637417193953826</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.4346025964147514</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2800</v>
+      </c>
+      <c r="C3" t="n">
+        <v>450</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-2.304957393348385</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.2811702192335956</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B4" t="n">
+        <v>3200</v>
+      </c>
+      <c r="C4" t="n">
+        <v>520</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-2.051605081387693</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.1530934413726104</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>35</v>
+      </c>
+      <c r="B5" t="n">
+        <v>4500</v>
+      </c>
+      <c r="C5" t="n">
+        <v>700</v>
+      </c>
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-1.694292205197514</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.1122001138223545</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>39</v>
+      </c>
+      <c r="B6" t="n">
+        <v>5200</v>
+      </c>
+      <c r="C6" t="n">
+        <v>850</v>
+      </c>
+      <c r="D6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-1.388796700952167</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.008531624239318792</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>42</v>
+      </c>
+      <c r="B7" t="n">
+        <v>6100</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1100</v>
+      </c>
+      <c r="D7" t="n">
+        <v>8</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-0.9989894608366757</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-0.05461118699078554</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>46</v>
+      </c>
+      <c r="B8" t="n">
+        <v>7500</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1250</v>
+      </c>
+      <c r="D8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-0.6471666286186903</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-0.08128390683026435</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>49</v>
+      </c>
+      <c r="B9" t="n">
+        <v>7500</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1400</v>
+      </c>
+      <c r="D9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-0.4215809384164558</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-0.2231836742363878</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>52</v>
+      </c>
+      <c r="B10" t="n">
+        <v>9800</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1700</v>
+      </c>
+      <c r="D10" t="n">
+        <v>12</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.08106134711526591</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-0.1377036327012556</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>55</v>
+      </c>
+      <c r="B11" t="n">
+        <v>11000</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2100</v>
+      </c>
+      <c r="D11" t="n">
+        <v>14</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.5512643247747445</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-0.1839543170640381</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>58</v>
+      </c>
+      <c r="B12" t="n">
+        <v>13500</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D12" t="n">
+        <v>16</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1.107503768669124</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-0.08721285761735803</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>61</v>
+      </c>
+      <c r="B13" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C13" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D13" t="n">
+        <v>18</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1.597561315459733</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-0.1004653549471876</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>64</v>
+      </c>
+      <c r="B14" t="n">
+        <v>7500</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3200</v>
+      </c>
+      <c r="D14" t="n">
+        <v>20</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1.451621009374509</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-1.09292608982185</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>68</v>
+      </c>
+      <c r="B15" t="n">
+        <v>21000</v>
+      </c>
+      <c r="C15" t="n">
+        <v>3800</v>
+      </c>
+      <c r="D15" t="n">
+        <v>24</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2.97875949252056</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.1345091924002882</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>72</v>
+      </c>
+      <c r="B16" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C16" t="n">
+        <v>4500</v>
+      </c>
+      <c r="D16" t="n">
+        <v>30</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4.377034344797472</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.8372338327262088</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Componente</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Variância_%</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Acumulada_%</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PC1</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>95.17</v>
+      </c>
+      <c r="C2" t="n">
+        <v>95.17</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PC2</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="C3" t="n">
+        <v>99.08</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PC3</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="C4" t="n">
+        <v>99.95999999999999</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PC4</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="C5" t="n">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2081,461 +2617,274 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Variável_X</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Variável_Y</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Correlação</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Fórmula_Excel</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Interpretação</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>Idade</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Renda_Mensal</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Estado_Civil</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
+      <c r="C2" t="n">
+        <v>0.9236</v>
+      </c>
+      <c r="D2">
+        <f>CORREL(Idade; Renda_Mensal)</f>
+        <v/>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Muito Forte</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Idade</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Valor_Compras</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="C3" t="n">
+        <v>0.9578</v>
+      </c>
+      <c r="D3">
+        <f>CORREL(Idade; Valor_Compras)</f>
+        <v/>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Muito Forte</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Idade</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Numero_Compras</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="C4" t="n">
+        <v>0.9614</v>
+      </c>
+      <c r="D4">
+        <f>CORREL(Idade; Numero_Compras)</f>
+        <v/>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Muito Forte</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Renda_Mensal</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Valor_Compras</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.986</v>
+      </c>
+      <c r="D5">
+        <f>CORREL(Renda_Mensal; Valor_Compras)</f>
+        <v/>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Muito Forte</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Renda_Mensal</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Numero_Compras</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.991</v>
+      </c>
+      <c r="D6">
+        <f>CORREL(Renda_Mensal; Numero_Compras)</f>
+        <v/>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Muito Forte</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Valor_Compras</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Numero_Compras</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.9976</v>
+      </c>
+      <c r="D7">
+        <f>CORREL(Valor_Compras; Numero_Compras)</f>
+        <v/>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Muito Forte</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Idade</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Classe</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Ticket_Medio</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Pct_Renda_Compras</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>22</v>
-      </c>
-      <c r="B2" t="n">
-        <v>2200</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Casado</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>300</v>
-      </c>
-      <c r="E2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>150</v>
-      </c>
-      <c r="H2" t="n">
-        <v>13.63636363636363</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>27</v>
-      </c>
-      <c r="B3" t="n">
-        <v>2800</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Casado</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>450</v>
-      </c>
-      <c r="E3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>150</v>
-      </c>
-      <c r="H3" t="n">
-        <v>16.07142857142857</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>31</v>
-      </c>
-      <c r="B4" t="n">
-        <v>3200</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Casado</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>520</v>
-      </c>
-      <c r="E4" t="n">
-        <v>4</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="n">
-        <v>130</v>
-      </c>
-      <c r="H4" t="n">
-        <v>16.25</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>35</v>
-      </c>
-      <c r="B5" t="n">
-        <v>4500</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Casado</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>700</v>
-      </c>
-      <c r="E5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
-        <v>140</v>
-      </c>
-      <c r="H5" t="n">
-        <v>15.55555555555556</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>39</v>
-      </c>
-      <c r="B6" t="n">
-        <v>5200</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Casado</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>850</v>
-      </c>
-      <c r="E6" t="n">
-        <v>6</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
-        <v>141.6666666666667</v>
-      </c>
-      <c r="H6" t="n">
-        <v>16.34615384615385</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>42</v>
-      </c>
-      <c r="B7" t="n">
-        <v>6100</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Casado</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1100</v>
-      </c>
-      <c r="E7" t="n">
-        <v>8</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" t="n">
-        <v>137.5</v>
-      </c>
-      <c r="H7" t="n">
-        <v>18.0327868852459</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>46</v>
-      </c>
-      <c r="B8" t="n">
-        <v>7500</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Casado</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>1250</v>
-      </c>
-      <c r="E8" t="n">
-        <v>9</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" t="n">
-        <v>138.8888888888889</v>
-      </c>
-      <c r="H8" t="n">
-        <v>16.66666666666666</v>
+      <c r="C8" t="n">
+        <v>0.8559</v>
+      </c>
+      <c r="D8">
+        <f>CORREL(Idade; Classe)</f>
+        <v/>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Forte</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>49</v>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Solteiro</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>1400</v>
-      </c>
-      <c r="E9" t="n">
-        <v>10</v>
-      </c>
-      <c r="F9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" t="n">
-        <v>140</v>
-      </c>
-      <c r="H9" t="inlineStr"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Renda_Mensal</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Classe</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.7799</v>
+      </c>
+      <c r="D9">
+        <f>CORREL(Renda_Mensal; Classe)</f>
+        <v/>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Forte</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>52</v>
-      </c>
-      <c r="B10" t="n">
-        <v>9800</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Casado</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>1700</v>
-      </c>
-      <c r="E10" t="n">
-        <v>12</v>
-      </c>
-      <c r="F10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" t="n">
-        <v>141.6666666666667</v>
-      </c>
-      <c r="H10" t="n">
-        <v>17.3469387755102</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Valor_Compras</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Classe</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.8012</v>
+      </c>
+      <c r="D10">
+        <f>CORREL(Valor_Compras; Classe)</f>
+        <v/>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Forte</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>55</v>
-      </c>
-      <c r="B11" t="n">
-        <v>11000</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Casado</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>2100</v>
-      </c>
-      <c r="E11" t="n">
-        <v>14</v>
-      </c>
-      <c r="F11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" t="n">
-        <v>150</v>
-      </c>
-      <c r="H11" t="n">
-        <v>19.09090909090909</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>58</v>
-      </c>
-      <c r="B12" t="n">
-        <v>13500</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Casado</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>2500</v>
-      </c>
-      <c r="E12" t="n">
-        <v>16</v>
-      </c>
-      <c r="F12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" t="n">
-        <v>156.25</v>
-      </c>
-      <c r="H12" t="n">
-        <v>18.51851851851852</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>61</v>
-      </c>
-      <c r="B13" t="n">
-        <v>15000</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Casado</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>2900</v>
-      </c>
-      <c r="E13" t="n">
-        <v>18</v>
-      </c>
-      <c r="F13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" t="n">
-        <v>161.1111111111111</v>
-      </c>
-      <c r="H13" t="n">
-        <v>19.33333333333333</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>64</v>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Casado</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>3200</v>
-      </c>
-      <c r="E14" t="n">
-        <v>20</v>
-      </c>
-      <c r="F14" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" t="n">
-        <v>160</v>
-      </c>
-      <c r="H14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>68</v>
-      </c>
-      <c r="B15" t="n">
-        <v>21000</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Casado</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>3800</v>
-      </c>
-      <c r="E15" t="n">
-        <v>24</v>
-      </c>
-      <c r="F15" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" t="n">
-        <v>158.3333333333333</v>
-      </c>
-      <c r="H15" t="n">
-        <v>18.09523809523809</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>72</v>
-      </c>
-      <c r="B16" t="n">
-        <v>30000</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Casado</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>4500</v>
-      </c>
-      <c r="E16" t="n">
-        <v>30</v>
-      </c>
-      <c r="F16" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" t="n">
-        <v>150</v>
-      </c>
-      <c r="H16" t="n">
-        <v>15</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Numero_Compras</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Classe</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.7983</v>
+      </c>
+      <c r="D11">
+        <f>CORREL(Numero_Compras; Classe)</f>
+        <v/>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Forte</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2549,285 +2898,105 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Idade</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Renda_Mensal</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Valor_Compras</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Numero_Compras</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Classe</t>
+          <t>Instruções para verificar no Excel</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>22</v>
-      </c>
-      <c r="B2" t="n">
-        <v>2200</v>
-      </c>
-      <c r="C2" t="n">
-        <v>300</v>
-      </c>
-      <c r="D2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Para calcular correlação no Excel, use:</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>27</v>
-      </c>
-      <c r="B3" t="n">
-        <v>2800</v>
-      </c>
-      <c r="C3" t="n">
-        <v>450</v>
-      </c>
-      <c r="D3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
+      <c r="A3">
+        <f>CORREL(A2:A16; B2:B16)</f>
+        <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>31</v>
-      </c>
-      <c r="B4" t="n">
-        <v>3200</v>
-      </c>
-      <c r="C4" t="n">
-        <v>520</v>
-      </c>
-      <c r="D4" t="n">
-        <v>4</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
+      <c r="A4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>35</v>
-      </c>
-      <c r="B5" t="n">
-        <v>4500</v>
-      </c>
-      <c r="C5" t="n">
-        <v>700</v>
-      </c>
-      <c r="D5" t="n">
-        <v>5</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Onde:</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>39</v>
-      </c>
-      <c r="B6" t="n">
-        <v>5200</v>
-      </c>
-      <c r="C6" t="n">
-        <v>850</v>
-      </c>
-      <c r="D6" t="n">
-        <v>6</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>A2:A16 = intervalo da primeira variável</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>42</v>
-      </c>
-      <c r="B7" t="n">
-        <v>6100</v>
-      </c>
-      <c r="C7" t="n">
-        <v>1100</v>
-      </c>
-      <c r="D7" t="n">
-        <v>8</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>B2:B16 = intervalo da segunda variável</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>46</v>
-      </c>
-      <c r="B8" t="n">
-        <v>7500</v>
-      </c>
-      <c r="C8" t="n">
-        <v>1250</v>
-      </c>
-      <c r="D8" t="n">
-        <v>9</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
+      <c r="A8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>49</v>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="n">
-        <v>1400</v>
-      </c>
-      <c r="D9" t="n">
-        <v>10</v>
-      </c>
-      <c r="E9" t="n">
-        <v>1</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Exemplo com os dados originais:</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>52</v>
-      </c>
-      <c r="B10" t="n">
-        <v>9800</v>
-      </c>
-      <c r="C10" t="n">
-        <v>1700</v>
-      </c>
-      <c r="D10" t="n">
-        <v>12</v>
-      </c>
-      <c r="E10" t="n">
-        <v>1</v>
+      <c r="A10">
+        <f>CORREL(A2:A16; D2:D16) para Idade vs Valor_Compras</f>
+        <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>55</v>
-      </c>
-      <c r="B11" t="n">
-        <v>11000</v>
-      </c>
-      <c r="C11" t="n">
-        <v>2100</v>
-      </c>
-      <c r="D11" t="n">
-        <v>14</v>
-      </c>
-      <c r="E11" t="n">
-        <v>1</v>
-      </c>
+      <c r="A11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="n">
-        <v>58</v>
-      </c>
-      <c r="B12" t="n">
-        <v>13500</v>
-      </c>
-      <c r="C12" t="n">
-        <v>2500</v>
-      </c>
-      <c r="D12" t="n">
-        <v>16</v>
-      </c>
-      <c r="E12" t="n">
-        <v>1</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Interpretação:</t>
+        </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
-        <v>61</v>
-      </c>
-      <c r="B13" t="n">
-        <v>15000</v>
-      </c>
-      <c r="C13" t="n">
-        <v>2900</v>
-      </c>
-      <c r="D13" t="n">
-        <v>18</v>
-      </c>
-      <c r="E13" t="n">
-        <v>1</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>&gt; 0.9 = Correlação Muito Forte</t>
+        </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
-        <v>64</v>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="n">
-        <v>3200</v>
-      </c>
-      <c r="D14" t="n">
-        <v>20</v>
-      </c>
-      <c r="E14" t="n">
-        <v>1</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>&gt; 0.7 = Correlação Forte</t>
+        </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
-        <v>68</v>
-      </c>
-      <c r="B15" t="n">
-        <v>21000</v>
-      </c>
-      <c r="C15" t="n">
-        <v>3800</v>
-      </c>
-      <c r="D15" t="n">
-        <v>24</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>&gt; 0.5 = Correlação Moderada</t>
+        </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
-        <v>72</v>
-      </c>
-      <c r="B16" t="n">
-        <v>30000</v>
-      </c>
-      <c r="C16" t="n">
-        <v>4500</v>
-      </c>
-      <c r="D16" t="n">
-        <v>30</v>
-      </c>
-      <c r="E16" t="n">
-        <v>1</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>&lt; 0.5 = Correlação Fraca</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2841,7 +3010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2857,22 +3026,32 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Estado_Civil</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Valor_Compras</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Numero_Compras</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Classe</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Imputado</t>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Ticket_Medio</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Pct_Renda_Compras</t>
         </is>
       </c>
     </row>
@@ -2883,19 +3062,25 @@
       <c r="B2" t="n">
         <v>2200</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
         <v>300</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>2</v>
       </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>150</v>
+      </c>
+      <c r="H2" t="n">
+        <v>13.63636363636363</v>
       </c>
     </row>
     <row r="3">
@@ -2905,19 +3090,25 @@
       <c r="B3" t="n">
         <v>2800</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
         <v>450</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>3</v>
       </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>150</v>
+      </c>
+      <c r="H3" t="n">
+        <v>16.07142857142857</v>
       </c>
     </row>
     <row r="4">
@@ -2927,19 +3118,25 @@
       <c r="B4" t="n">
         <v>3200</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
         <v>520</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>4</v>
       </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>130</v>
+      </c>
+      <c r="H4" t="n">
+        <v>16.25</v>
       </c>
     </row>
     <row r="5">
@@ -2949,19 +3146,25 @@
       <c r="B5" t="n">
         <v>4500</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
         <v>700</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>5</v>
       </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>140</v>
+      </c>
+      <c r="H5" t="n">
+        <v>15.55555555555556</v>
       </c>
     </row>
     <row r="6">
@@ -2971,19 +3174,25 @@
       <c r="B6" t="n">
         <v>5200</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
         <v>850</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>6</v>
       </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>141.6666666666667</v>
+      </c>
+      <c r="H6" t="n">
+        <v>16.34615384615385</v>
       </c>
     </row>
     <row r="7">
@@ -2993,19 +3202,25 @@
       <c r="B7" t="n">
         <v>6100</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
         <v>1100</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>8</v>
       </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>137.5</v>
+      </c>
+      <c r="H7" t="n">
+        <v>18.0327868852459</v>
       </c>
     </row>
     <row r="8">
@@ -3015,42 +3230,50 @@
       <c r="B8" t="n">
         <v>7500</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
         <v>1250</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>9</v>
       </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>138.8888888888889</v>
+      </c>
+      <c r="H8" t="n">
+        <v>16.66666666666666</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
         <v>49</v>
       </c>
-      <c r="B9" t="n">
-        <v>7500</v>
-      </c>
-      <c r="C9" t="n">
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
         <v>1400</v>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="n">
         <v>10</v>
       </c>
-      <c r="E9" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>140</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -3059,19 +3282,25 @@
       <c r="B10" t="n">
         <v>9800</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
         <v>1700</v>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
         <v>12</v>
       </c>
-      <c r="E10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>141.6666666666667</v>
+      </c>
+      <c r="H10" t="n">
+        <v>17.3469387755102</v>
       </c>
     </row>
     <row r="11">
@@ -3081,19 +3310,25 @@
       <c r="B11" t="n">
         <v>11000</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
         <v>2100</v>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>14</v>
       </c>
-      <c r="E11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>150</v>
+      </c>
+      <c r="H11" t="n">
+        <v>19.09090909090909</v>
       </c>
     </row>
     <row r="12">
@@ -3103,19 +3338,25 @@
       <c r="B12" t="n">
         <v>13500</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
         <v>2500</v>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
         <v>16</v>
       </c>
-      <c r="E12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="n">
+        <v>156.25</v>
+      </c>
+      <c r="H12" t="n">
+        <v>18.51851851851852</v>
       </c>
     </row>
     <row r="13">
@@ -3125,42 +3366,50 @@
       <c r="B13" t="n">
         <v>15000</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
         <v>2900</v>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="n">
         <v>18</v>
       </c>
-      <c r="E13" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="n">
+        <v>161.1111111111111</v>
+      </c>
+      <c r="H13" t="n">
+        <v>19.33333333333333</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
         <v>64</v>
       </c>
-      <c r="B14" t="n">
-        <v>7500</v>
-      </c>
-      <c r="C14" t="n">
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
         <v>3200</v>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="n">
         <v>20</v>
       </c>
-      <c r="E14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="n">
+        <v>160</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -3169,19 +3418,25 @@
       <c r="B15" t="n">
         <v>21000</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
         <v>3800</v>
       </c>
-      <c r="D15" t="n">
+      <c r="E15" t="n">
         <v>24</v>
       </c>
-      <c r="E15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="n">
+        <v>158.3333333333333</v>
+      </c>
+      <c r="H15" t="n">
+        <v>18.09523809523809</v>
       </c>
     </row>
     <row r="16">
@@ -3191,19 +3446,25 @@
       <c r="B16" t="n">
         <v>30000</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
         <v>4500</v>
       </c>
-      <c r="D16" t="n">
+      <c r="E16" t="n">
         <v>30</v>
       </c>
-      <c r="E16" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="n">
+        <v>150</v>
+      </c>
+      <c r="H16" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -3217,7 +3478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3246,21 +3507,6 @@
           <t>Classe</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Log_Renda</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Faixa_Idade</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Faixa_Renda</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -3278,19 +3524,6 @@
       <c r="E2" t="n">
         <v>0</v>
       </c>
-      <c r="F2" t="n">
-        <v>7.696212639346407</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Jovem</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Baixa</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -3308,19 +3541,6 @@
       <c r="E3" t="n">
         <v>0</v>
       </c>
-      <c r="F3" t="n">
-        <v>7.937374696163295</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Jovem</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Baixa</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -3338,19 +3558,6 @@
       <c r="E4" t="n">
         <v>0</v>
       </c>
-      <c r="F4" t="n">
-        <v>8.070906088787819</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Jovem</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Baixa</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -3368,19 +3575,6 @@
       <c r="E5" t="n">
         <v>0</v>
       </c>
-      <c r="F5" t="n">
-        <v>8.411832675758411</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Jovem</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -3398,19 +3592,6 @@
       <c r="E6" t="n">
         <v>0</v>
       </c>
-      <c r="F6" t="n">
-        <v>8.556413904569519</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Adulto</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -3428,19 +3609,6 @@
       <c r="E7" t="n">
         <v>0</v>
       </c>
-      <c r="F7" t="n">
-        <v>8.716044050161402</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Adulto</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -3458,27 +3626,12 @@
       <c r="E8" t="n">
         <v>0</v>
       </c>
-      <c r="F8" t="n">
-        <v>8.922658299524402</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Adulto</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
         <v>49</v>
       </c>
-      <c r="B9" t="n">
-        <v>7500</v>
-      </c>
+      <c r="B9" t="inlineStr"/>
       <c r="C9" t="n">
         <v>1400</v>
       </c>
@@ -3487,19 +3640,6 @@
       </c>
       <c r="E9" t="n">
         <v>1</v>
-      </c>
-      <c r="F9" t="n">
-        <v>8.922658299524402</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Adulto</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
       </c>
     </row>
     <row r="10">
@@ -3518,19 +3658,6 @@
       <c r="E10" t="n">
         <v>1</v>
       </c>
-      <c r="F10" t="n">
-        <v>9.190137664658664</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Maduro</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -3548,19 +3675,6 @@
       <c r="E11" t="n">
         <v>1</v>
       </c>
-      <c r="F11" t="n">
-        <v>9.305650551780507</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Maduro</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -3578,19 +3692,6 @@
       <c r="E12" t="n">
         <v>1</v>
       </c>
-      <c r="F12" t="n">
-        <v>9.510444964426521</v>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Maduro</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -3608,27 +3709,12 @@
       <c r="E13" t="n">
         <v>1</v>
       </c>
-      <c r="F13" t="n">
-        <v>9.615805480084347</v>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Maduro</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
         <v>64</v>
       </c>
-      <c r="B14" t="n">
-        <v>7500</v>
-      </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
         <v>3200</v>
       </c>
@@ -3637,19 +3723,6 @@
       </c>
       <c r="E14" t="n">
         <v>1</v>
-      </c>
-      <c r="F14" t="n">
-        <v>8.922658299524402</v>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Maduro</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
       </c>
     </row>
     <row r="15">
@@ -3668,19 +3741,6 @@
       <c r="E15" t="n">
         <v>1</v>
       </c>
-      <c r="F15" t="n">
-        <v>9.952277716705559</v>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Muito_Alta</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -3697,19 +3757,6 @@
       </c>
       <c r="E16" t="n">
         <v>1</v>
-      </c>
-      <c r="F16" t="n">
-        <v>10.30895266064429</v>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Muito_Alta</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -3723,7 +3770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3754,12 +3801,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>EC_Casado</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>EC_Solteiro</t>
+          <t>Imputado</t>
         </is>
       </c>
     </row>
@@ -3779,11 +3821,10 @@
       <c r="E2" t="n">
         <v>0</v>
       </c>
-      <c r="F2" t="b">
-        <v>1</v>
-      </c>
-      <c r="G2" t="b">
-        <v>0</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -3802,11 +3843,10 @@
       <c r="E3" t="n">
         <v>0</v>
       </c>
-      <c r="F3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G3" t="b">
-        <v>0</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -3825,11 +3865,10 @@
       <c r="E4" t="n">
         <v>0</v>
       </c>
-      <c r="F4" t="b">
-        <v>1</v>
-      </c>
-      <c r="G4" t="b">
-        <v>0</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -3848,11 +3887,10 @@
       <c r="E5" t="n">
         <v>0</v>
       </c>
-      <c r="F5" t="b">
-        <v>1</v>
-      </c>
-      <c r="G5" t="b">
-        <v>0</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -3871,11 +3909,10 @@
       <c r="E6" t="n">
         <v>0</v>
       </c>
-      <c r="F6" t="b">
-        <v>1</v>
-      </c>
-      <c r="G6" t="b">
-        <v>0</v>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -3894,11 +3931,10 @@
       <c r="E7" t="n">
         <v>0</v>
       </c>
-      <c r="F7" t="b">
-        <v>1</v>
-      </c>
-      <c r="G7" t="b">
-        <v>0</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -3917,18 +3953,19 @@
       <c r="E8" t="n">
         <v>0</v>
       </c>
-      <c r="F8" t="b">
-        <v>1</v>
-      </c>
-      <c r="G8" t="b">
-        <v>0</v>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
         <v>49</v>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="n">
+        <v>7500</v>
+      </c>
       <c r="C9" t="n">
         <v>1400</v>
       </c>
@@ -3938,11 +3975,10 @@
       <c r="E9" t="n">
         <v>1</v>
       </c>
-      <c r="F9" t="b">
-        <v>0</v>
-      </c>
-      <c r="G9" t="b">
-        <v>1</v>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -3961,11 +3997,10 @@
       <c r="E10" t="n">
         <v>1</v>
       </c>
-      <c r="F10" t="b">
-        <v>1</v>
-      </c>
-      <c r="G10" t="b">
-        <v>0</v>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -3984,11 +4019,10 @@
       <c r="E11" t="n">
         <v>1</v>
       </c>
-      <c r="F11" t="b">
-        <v>1</v>
-      </c>
-      <c r="G11" t="b">
-        <v>0</v>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -4007,11 +4041,10 @@
       <c r="E12" t="n">
         <v>1</v>
       </c>
-      <c r="F12" t="b">
-        <v>1</v>
-      </c>
-      <c r="G12" t="b">
-        <v>0</v>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -4030,18 +4063,19 @@
       <c r="E13" t="n">
         <v>1</v>
       </c>
-      <c r="F13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G13" t="b">
-        <v>0</v>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
         <v>64</v>
       </c>
-      <c r="B14" t="inlineStr"/>
+      <c r="B14" t="n">
+        <v>7500</v>
+      </c>
       <c r="C14" t="n">
         <v>3200</v>
       </c>
@@ -4051,11 +4085,10 @@
       <c r="E14" t="n">
         <v>1</v>
       </c>
-      <c r="F14" t="b">
-        <v>1</v>
-      </c>
-      <c r="G14" t="b">
-        <v>0</v>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -4074,11 +4107,10 @@
       <c r="E15" t="n">
         <v>1</v>
       </c>
-      <c r="F15" t="b">
-        <v>1</v>
-      </c>
-      <c r="G15" t="b">
-        <v>0</v>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -4097,11 +4129,10 @@
       <c r="E16" t="n">
         <v>1</v>
       </c>
-      <c r="F16" t="b">
-        <v>1</v>
-      </c>
-      <c r="G16" t="b">
-        <v>0</v>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -4115,134 +4146,498 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Variável</t>
+          <t>Idade</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Média_Classe_0</t>
+          <t>Renda_Mensal</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Média_Classe_1</t>
+          <t>Valor_Compras</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>F_Statistic</t>
+          <t>Numero_Compras</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>P_Value</t>
+          <t>Classe</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Significativo</t>
+          <t>Log_Renda</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Faixa_Idade</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Faixa_Renda</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Idade</t>
-        </is>
+      <c r="A2" t="n">
+        <v>22</v>
       </c>
       <c r="B2" t="n">
-        <v>34.57</v>
+        <v>2200</v>
       </c>
       <c r="C2" t="n">
-        <v>59.88</v>
+        <v>300</v>
       </c>
       <c r="D2" t="n">
-        <v>35.6118</v>
+        <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>4.7e-05</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Sim</t>
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>7.696212639346407</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Jovem</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Baixa</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Renda_Mensal</t>
-        </is>
+      <c r="A3" t="n">
+        <v>27</v>
       </c>
       <c r="B3" t="n">
+        <v>2800</v>
+      </c>
+      <c r="C3" t="n">
+        <v>450</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>7.937374696163295</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Jovem</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Baixa</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B4" t="n">
+        <v>3200</v>
+      </c>
+      <c r="C4" t="n">
+        <v>520</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>8.070906088787819</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Jovem</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Baixa</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>35</v>
+      </c>
+      <c r="B5" t="n">
         <v>4500</v>
       </c>
-      <c r="C3" t="n">
-        <v>14412.5</v>
-      </c>
-      <c r="D3" t="n">
-        <v>10.8889</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.00575</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Valor_Compras</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>738.5700000000001</v>
-      </c>
-      <c r="C4" t="n">
-        <v>2762.5</v>
-      </c>
-      <c r="D4" t="n">
-        <v>23.3116</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.00033</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Numero_Compras</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>5.29</v>
-      </c>
       <c r="C5" t="n">
+        <v>700</v>
+      </c>
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>8.411832675758411</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Jovem</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>39</v>
+      </c>
+      <c r="B6" t="n">
+        <v>5200</v>
+      </c>
+      <c r="C6" t="n">
+        <v>850</v>
+      </c>
+      <c r="D6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>8.556413904569519</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Adulto</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>42</v>
+      </c>
+      <c r="B7" t="n">
+        <v>6100</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1100</v>
+      </c>
+      <c r="D7" t="n">
+        <v>8</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>8.716044050161402</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Adulto</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>46</v>
+      </c>
+      <c r="B8" t="n">
+        <v>7500</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1250</v>
+      </c>
+      <c r="D8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>8.922658299524402</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Adulto</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>49</v>
+      </c>
+      <c r="B9" t="n">
+        <v>7500</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1400</v>
+      </c>
+      <c r="D9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>8.922658299524402</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Adulto</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>52</v>
+      </c>
+      <c r="B10" t="n">
+        <v>9800</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1700</v>
+      </c>
+      <c r="D10" t="n">
+        <v>12</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>9.190137664658664</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Maduro</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>55</v>
+      </c>
+      <c r="B11" t="n">
+        <v>11000</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2100</v>
+      </c>
+      <c r="D11" t="n">
+        <v>14</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>9.305650551780507</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Maduro</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>58</v>
+      </c>
+      <c r="B12" t="n">
+        <v>13500</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D12" t="n">
+        <v>16</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>9.510444964426521</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Maduro</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>61</v>
+      </c>
+      <c r="B13" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C13" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D13" t="n">
         <v>18</v>
       </c>
-      <c r="D5" t="n">
-        <v>22.8448</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.00036</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>9.615805480084347</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Maduro</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>64</v>
+      </c>
+      <c r="B14" t="n">
+        <v>7500</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3200</v>
+      </c>
+      <c r="D14" t="n">
+        <v>20</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>8.922658299524402</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Maduro</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>68</v>
+      </c>
+      <c r="B15" t="n">
+        <v>21000</v>
+      </c>
+      <c r="C15" t="n">
+        <v>3800</v>
+      </c>
+      <c r="D15" t="n">
+        <v>24</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>9.952277716705559</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Muito_Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>72</v>
+      </c>
+      <c r="B16" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C16" t="n">
+        <v>4500</v>
+      </c>
+      <c r="D16" t="n">
+        <v>30</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>10.30895266064429</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Muito_Alta</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Detalha passo 1.6 com todas as transformações
Colunas adicionadas:
- Log_Renda: =LN(B2)
- Faixa_Idade: =SE(A2<=35;"Jovem";SE(...))
- Faixa_Renda: =SE(B2<=4000;"Baixa";SE(...))
- Faixa_Valor: =SE(C2<=500;"Baixo";SE(...))
- Renda_Normalizada: Min-Max scaling

Inclui explicações detalhadas das fórmulas
</commit_message>
<xml_diff>
--- a/dados/Dados_Tratados_Exercicios.xlsx
+++ b/dados/Dados_Tratados_Exercicios.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados Originais" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados Tratados" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="passo 1.5" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="passo 1.6" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,13 +31,23 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDDDDD"/>
+        <bgColor rgb="00DDDDDD"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -51,9 +62,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1974,4 +1987,941 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Idade</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Renda_Mensal</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Valor_Compras</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Numero_Compras</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Classe</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Log_Renda</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Faixa_Idade</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Faixa_Renda</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Faixa_Valor</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Renda_Normalizada</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <f>'Dados Tratados'!A2</f>
+        <v/>
+      </c>
+      <c r="B2">
+        <f>'Dados Tratados'!B2</f>
+        <v/>
+      </c>
+      <c r="C2">
+        <f>'Dados Tratados'!C2</f>
+        <v/>
+      </c>
+      <c r="D2">
+        <f>'Dados Tratados'!D2</f>
+        <v/>
+      </c>
+      <c r="E2">
+        <f>'Dados Tratados'!E2</f>
+        <v/>
+      </c>
+      <c r="F2">
+        <f>LN(B2)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>SE(A2&lt;=35;"Jovem";SE(A2&lt;=50;"Adulto";SE(A2&lt;=65;"Maduro";"Senior")))</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>SE(B2&lt;=4000;"Baixa";SE(B2&lt;=8000;"Media";SE(B2&lt;=15000;"Alta";"Muito_Alta")))</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>SE(C2&lt;=500;"Baixo";SE(C2&lt;=1500;"Medio";SE(C2&lt;=3000;"Alto";"Muito_Alto")))</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>(B2-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <f>'Dados Tratados'!A3</f>
+        <v/>
+      </c>
+      <c r="B3">
+        <f>'Dados Tratados'!B3</f>
+        <v/>
+      </c>
+      <c r="C3">
+        <f>'Dados Tratados'!C3</f>
+        <v/>
+      </c>
+      <c r="D3">
+        <f>'Dados Tratados'!D3</f>
+        <v/>
+      </c>
+      <c r="E3">
+        <f>'Dados Tratados'!E3</f>
+        <v/>
+      </c>
+      <c r="F3">
+        <f>LN(B3)</f>
+        <v/>
+      </c>
+      <c r="G3">
+        <f>SE(A3&lt;=35;"Jovem";SE(A3&lt;=50;"Adulto";SE(A3&lt;=65;"Maduro";"Senior")))</f>
+        <v/>
+      </c>
+      <c r="H3">
+        <f>SE(B3&lt;=4000;"Baixa";SE(B3&lt;=8000;"Media";SE(B3&lt;=15000;"Alta";"Muito_Alta")))</f>
+        <v/>
+      </c>
+      <c r="I3">
+        <f>SE(C3&lt;=500;"Baixo";SE(C3&lt;=1500;"Medio";SE(C3&lt;=3000;"Alto";"Muito_Alto")))</f>
+        <v/>
+      </c>
+      <c r="J3">
+        <f>(B3-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <f>'Dados Tratados'!A4</f>
+        <v/>
+      </c>
+      <c r="B4">
+        <f>'Dados Tratados'!B4</f>
+        <v/>
+      </c>
+      <c r="C4">
+        <f>'Dados Tratados'!C4</f>
+        <v/>
+      </c>
+      <c r="D4">
+        <f>'Dados Tratados'!D4</f>
+        <v/>
+      </c>
+      <c r="E4">
+        <f>'Dados Tratados'!E4</f>
+        <v/>
+      </c>
+      <c r="F4">
+        <f>LN(B4)</f>
+        <v/>
+      </c>
+      <c r="G4">
+        <f>SE(A4&lt;=35;"Jovem";SE(A4&lt;=50;"Adulto";SE(A4&lt;=65;"Maduro";"Senior")))</f>
+        <v/>
+      </c>
+      <c r="H4">
+        <f>SE(B4&lt;=4000;"Baixa";SE(B4&lt;=8000;"Media";SE(B4&lt;=15000;"Alta";"Muito_Alta")))</f>
+        <v/>
+      </c>
+      <c r="I4">
+        <f>SE(C4&lt;=500;"Baixo";SE(C4&lt;=1500;"Medio";SE(C4&lt;=3000;"Alto";"Muito_Alto")))</f>
+        <v/>
+      </c>
+      <c r="J4">
+        <f>(B4-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <f>'Dados Tratados'!A5</f>
+        <v/>
+      </c>
+      <c r="B5">
+        <f>'Dados Tratados'!B5</f>
+        <v/>
+      </c>
+      <c r="C5">
+        <f>'Dados Tratados'!C5</f>
+        <v/>
+      </c>
+      <c r="D5">
+        <f>'Dados Tratados'!D5</f>
+        <v/>
+      </c>
+      <c r="E5">
+        <f>'Dados Tratados'!E5</f>
+        <v/>
+      </c>
+      <c r="F5">
+        <f>LN(B5)</f>
+        <v/>
+      </c>
+      <c r="G5">
+        <f>SE(A5&lt;=35;"Jovem";SE(A5&lt;=50;"Adulto";SE(A5&lt;=65;"Maduro";"Senior")))</f>
+        <v/>
+      </c>
+      <c r="H5">
+        <f>SE(B5&lt;=4000;"Baixa";SE(B5&lt;=8000;"Media";SE(B5&lt;=15000;"Alta";"Muito_Alta")))</f>
+        <v/>
+      </c>
+      <c r="I5">
+        <f>SE(C5&lt;=500;"Baixo";SE(C5&lt;=1500;"Medio";SE(C5&lt;=3000;"Alto";"Muito_Alto")))</f>
+        <v/>
+      </c>
+      <c r="J5">
+        <f>(B5-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <f>'Dados Tratados'!A6</f>
+        <v/>
+      </c>
+      <c r="B6">
+        <f>'Dados Tratados'!B6</f>
+        <v/>
+      </c>
+      <c r="C6">
+        <f>'Dados Tratados'!C6</f>
+        <v/>
+      </c>
+      <c r="D6">
+        <f>'Dados Tratados'!D6</f>
+        <v/>
+      </c>
+      <c r="E6">
+        <f>'Dados Tratados'!E6</f>
+        <v/>
+      </c>
+      <c r="F6">
+        <f>LN(B6)</f>
+        <v/>
+      </c>
+      <c r="G6">
+        <f>SE(A6&lt;=35;"Jovem";SE(A6&lt;=50;"Adulto";SE(A6&lt;=65;"Maduro";"Senior")))</f>
+        <v/>
+      </c>
+      <c r="H6">
+        <f>SE(B6&lt;=4000;"Baixa";SE(B6&lt;=8000;"Media";SE(B6&lt;=15000;"Alta";"Muito_Alta")))</f>
+        <v/>
+      </c>
+      <c r="I6">
+        <f>SE(C6&lt;=500;"Baixo";SE(C6&lt;=1500;"Medio";SE(C6&lt;=3000;"Alto";"Muito_Alto")))</f>
+        <v/>
+      </c>
+      <c r="J6">
+        <f>(B6-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <f>'Dados Tratados'!A7</f>
+        <v/>
+      </c>
+      <c r="B7">
+        <f>'Dados Tratados'!B7</f>
+        <v/>
+      </c>
+      <c r="C7">
+        <f>'Dados Tratados'!C7</f>
+        <v/>
+      </c>
+      <c r="D7">
+        <f>'Dados Tratados'!D7</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>'Dados Tratados'!E7</f>
+        <v/>
+      </c>
+      <c r="F7">
+        <f>LN(B7)</f>
+        <v/>
+      </c>
+      <c r="G7">
+        <f>SE(A7&lt;=35;"Jovem";SE(A7&lt;=50;"Adulto";SE(A7&lt;=65;"Maduro";"Senior")))</f>
+        <v/>
+      </c>
+      <c r="H7">
+        <f>SE(B7&lt;=4000;"Baixa";SE(B7&lt;=8000;"Media";SE(B7&lt;=15000;"Alta";"Muito_Alta")))</f>
+        <v/>
+      </c>
+      <c r="I7">
+        <f>SE(C7&lt;=500;"Baixo";SE(C7&lt;=1500;"Medio";SE(C7&lt;=3000;"Alto";"Muito_Alto")))</f>
+        <v/>
+      </c>
+      <c r="J7">
+        <f>(B7-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <f>'Dados Tratados'!A8</f>
+        <v/>
+      </c>
+      <c r="B8">
+        <f>'Dados Tratados'!B8</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>'Dados Tratados'!C8</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>'Dados Tratados'!D8</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>'Dados Tratados'!E8</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>LN(B8)</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>SE(A8&lt;=35;"Jovem";SE(A8&lt;=50;"Adulto";SE(A8&lt;=65;"Maduro";"Senior")))</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>SE(B8&lt;=4000;"Baixa";SE(B8&lt;=8000;"Media";SE(B8&lt;=15000;"Alta";"Muito_Alta")))</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>SE(C8&lt;=500;"Baixo";SE(C8&lt;=1500;"Medio";SE(C8&lt;=3000;"Alto";"Muito_Alto")))</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>(B8-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <f>'Dados Tratados'!A9</f>
+        <v/>
+      </c>
+      <c r="B9">
+        <f>'Dados Tratados'!B9</f>
+        <v/>
+      </c>
+      <c r="C9">
+        <f>'Dados Tratados'!C9</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>'Dados Tratados'!D9</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>'Dados Tratados'!E9</f>
+        <v/>
+      </c>
+      <c r="F9">
+        <f>LN(B9)</f>
+        <v/>
+      </c>
+      <c r="G9">
+        <f>SE(A9&lt;=35;"Jovem";SE(A9&lt;=50;"Adulto";SE(A9&lt;=65;"Maduro";"Senior")))</f>
+        <v/>
+      </c>
+      <c r="H9">
+        <f>SE(B9&lt;=4000;"Baixa";SE(B9&lt;=8000;"Media";SE(B9&lt;=15000;"Alta";"Muito_Alta")))</f>
+        <v/>
+      </c>
+      <c r="I9">
+        <f>SE(C9&lt;=500;"Baixo";SE(C9&lt;=1500;"Medio";SE(C9&lt;=3000;"Alto";"Muito_Alto")))</f>
+        <v/>
+      </c>
+      <c r="J9">
+        <f>(B9-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <f>'Dados Tratados'!A10</f>
+        <v/>
+      </c>
+      <c r="B10">
+        <f>'Dados Tratados'!B10</f>
+        <v/>
+      </c>
+      <c r="C10">
+        <f>'Dados Tratados'!C10</f>
+        <v/>
+      </c>
+      <c r="D10">
+        <f>'Dados Tratados'!D10</f>
+        <v/>
+      </c>
+      <c r="E10">
+        <f>'Dados Tratados'!E10</f>
+        <v/>
+      </c>
+      <c r="F10">
+        <f>LN(B10)</f>
+        <v/>
+      </c>
+      <c r="G10">
+        <f>SE(A10&lt;=35;"Jovem";SE(A10&lt;=50;"Adulto";SE(A10&lt;=65;"Maduro";"Senior")))</f>
+        <v/>
+      </c>
+      <c r="H10">
+        <f>SE(B10&lt;=4000;"Baixa";SE(B10&lt;=8000;"Media";SE(B10&lt;=15000;"Alta";"Muito_Alta")))</f>
+        <v/>
+      </c>
+      <c r="I10">
+        <f>SE(C10&lt;=500;"Baixo";SE(C10&lt;=1500;"Medio";SE(C10&lt;=3000;"Alto";"Muito_Alto")))</f>
+        <v/>
+      </c>
+      <c r="J10">
+        <f>(B10-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <f>'Dados Tratados'!A11</f>
+        <v/>
+      </c>
+      <c r="B11">
+        <f>'Dados Tratados'!B11</f>
+        <v/>
+      </c>
+      <c r="C11">
+        <f>'Dados Tratados'!C11</f>
+        <v/>
+      </c>
+      <c r="D11">
+        <f>'Dados Tratados'!D11</f>
+        <v/>
+      </c>
+      <c r="E11">
+        <f>'Dados Tratados'!E11</f>
+        <v/>
+      </c>
+      <c r="F11">
+        <f>LN(B11)</f>
+        <v/>
+      </c>
+      <c r="G11">
+        <f>SE(A11&lt;=35;"Jovem";SE(A11&lt;=50;"Adulto";SE(A11&lt;=65;"Maduro";"Senior")))</f>
+        <v/>
+      </c>
+      <c r="H11">
+        <f>SE(B11&lt;=4000;"Baixa";SE(B11&lt;=8000;"Media";SE(B11&lt;=15000;"Alta";"Muito_Alta")))</f>
+        <v/>
+      </c>
+      <c r="I11">
+        <f>SE(C11&lt;=500;"Baixo";SE(C11&lt;=1500;"Medio";SE(C11&lt;=3000;"Alto";"Muito_Alto")))</f>
+        <v/>
+      </c>
+      <c r="J11">
+        <f>(B11-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <f>'Dados Tratados'!A12</f>
+        <v/>
+      </c>
+      <c r="B12">
+        <f>'Dados Tratados'!B12</f>
+        <v/>
+      </c>
+      <c r="C12">
+        <f>'Dados Tratados'!C12</f>
+        <v/>
+      </c>
+      <c r="D12">
+        <f>'Dados Tratados'!D12</f>
+        <v/>
+      </c>
+      <c r="E12">
+        <f>'Dados Tratados'!E12</f>
+        <v/>
+      </c>
+      <c r="F12">
+        <f>LN(B12)</f>
+        <v/>
+      </c>
+      <c r="G12">
+        <f>SE(A12&lt;=35;"Jovem";SE(A12&lt;=50;"Adulto";SE(A12&lt;=65;"Maduro";"Senior")))</f>
+        <v/>
+      </c>
+      <c r="H12">
+        <f>SE(B12&lt;=4000;"Baixa";SE(B12&lt;=8000;"Media";SE(B12&lt;=15000;"Alta";"Muito_Alta")))</f>
+        <v/>
+      </c>
+      <c r="I12">
+        <f>SE(C12&lt;=500;"Baixo";SE(C12&lt;=1500;"Medio";SE(C12&lt;=3000;"Alto";"Muito_Alto")))</f>
+        <v/>
+      </c>
+      <c r="J12">
+        <f>(B12-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <f>'Dados Tratados'!A13</f>
+        <v/>
+      </c>
+      <c r="B13">
+        <f>'Dados Tratados'!B13</f>
+        <v/>
+      </c>
+      <c r="C13">
+        <f>'Dados Tratados'!C13</f>
+        <v/>
+      </c>
+      <c r="D13">
+        <f>'Dados Tratados'!D13</f>
+        <v/>
+      </c>
+      <c r="E13">
+        <f>'Dados Tratados'!E13</f>
+        <v/>
+      </c>
+      <c r="F13">
+        <f>LN(B13)</f>
+        <v/>
+      </c>
+      <c r="G13">
+        <f>SE(A13&lt;=35;"Jovem";SE(A13&lt;=50;"Adulto";SE(A13&lt;=65;"Maduro";"Senior")))</f>
+        <v/>
+      </c>
+      <c r="H13">
+        <f>SE(B13&lt;=4000;"Baixa";SE(B13&lt;=8000;"Media";SE(B13&lt;=15000;"Alta";"Muito_Alta")))</f>
+        <v/>
+      </c>
+      <c r="I13">
+        <f>SE(C13&lt;=500;"Baixo";SE(C13&lt;=1500;"Medio";SE(C13&lt;=3000;"Alto";"Muito_Alto")))</f>
+        <v/>
+      </c>
+      <c r="J13">
+        <f>(B13-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <f>'Dados Tratados'!A14</f>
+        <v/>
+      </c>
+      <c r="B14">
+        <f>'Dados Tratados'!B14</f>
+        <v/>
+      </c>
+      <c r="C14">
+        <f>'Dados Tratados'!C14</f>
+        <v/>
+      </c>
+      <c r="D14">
+        <f>'Dados Tratados'!D14</f>
+        <v/>
+      </c>
+      <c r="E14">
+        <f>'Dados Tratados'!E14</f>
+        <v/>
+      </c>
+      <c r="F14">
+        <f>LN(B14)</f>
+        <v/>
+      </c>
+      <c r="G14">
+        <f>SE(A14&lt;=35;"Jovem";SE(A14&lt;=50;"Adulto";SE(A14&lt;=65;"Maduro";"Senior")))</f>
+        <v/>
+      </c>
+      <c r="H14">
+        <f>SE(B14&lt;=4000;"Baixa";SE(B14&lt;=8000;"Media";SE(B14&lt;=15000;"Alta";"Muito_Alta")))</f>
+        <v/>
+      </c>
+      <c r="I14">
+        <f>SE(C14&lt;=500;"Baixo";SE(C14&lt;=1500;"Medio";SE(C14&lt;=3000;"Alto";"Muito_Alto")))</f>
+        <v/>
+      </c>
+      <c r="J14">
+        <f>(B14-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <f>'Dados Tratados'!A15</f>
+        <v/>
+      </c>
+      <c r="B15">
+        <f>'Dados Tratados'!B15</f>
+        <v/>
+      </c>
+      <c r="C15">
+        <f>'Dados Tratados'!C15</f>
+        <v/>
+      </c>
+      <c r="D15">
+        <f>'Dados Tratados'!D15</f>
+        <v/>
+      </c>
+      <c r="E15">
+        <f>'Dados Tratados'!E15</f>
+        <v/>
+      </c>
+      <c r="F15">
+        <f>LN(B15)</f>
+        <v/>
+      </c>
+      <c r="G15">
+        <f>SE(A15&lt;=35;"Jovem";SE(A15&lt;=50;"Adulto";SE(A15&lt;=65;"Maduro";"Senior")))</f>
+        <v/>
+      </c>
+      <c r="H15">
+        <f>SE(B15&lt;=4000;"Baixa";SE(B15&lt;=8000;"Media";SE(B15&lt;=15000;"Alta";"Muito_Alta")))</f>
+        <v/>
+      </c>
+      <c r="I15">
+        <f>SE(C15&lt;=500;"Baixo";SE(C15&lt;=1500;"Medio";SE(C15&lt;=3000;"Alto";"Muito_Alto")))</f>
+        <v/>
+      </c>
+      <c r="J15">
+        <f>(B15-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <f>'Dados Tratados'!A16</f>
+        <v/>
+      </c>
+      <c r="B16">
+        <f>'Dados Tratados'!B16</f>
+        <v/>
+      </c>
+      <c r="C16">
+        <f>'Dados Tratados'!C16</f>
+        <v/>
+      </c>
+      <c r="D16">
+        <f>'Dados Tratados'!D16</f>
+        <v/>
+      </c>
+      <c r="E16">
+        <f>'Dados Tratados'!E16</f>
+        <v/>
+      </c>
+      <c r="F16">
+        <f>LN(B16)</f>
+        <v/>
+      </c>
+      <c r="G16">
+        <f>SE(A16&lt;=35;"Jovem";SE(A16&lt;=50;"Adulto";SE(A16&lt;=65;"Maduro";"Senior")))</f>
+        <v/>
+      </c>
+      <c r="H16">
+        <f>SE(B16&lt;=4000;"Baixa";SE(B16&lt;=8000;"Media";SE(B16&lt;=15000;"Alta";"Muito_Alta")))</f>
+        <v/>
+      </c>
+      <c r="I16">
+        <f>SE(C16&lt;=500;"Baixo";SE(C16&lt;=1500;"Medio";SE(C16&lt;=3000;"Alto";"Muito_Alto")))</f>
+        <v/>
+      </c>
+      <c r="J16">
+        <f>(B16-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3">
+        <f>== EXPLICAÇÃO DAS TRANSFORMAÇÕES ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>1. LOG_RENDA (Coluna F)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Fórmula: =LN(B2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Por quê: Renda tem amplitude muito grande (2200 a 30000 = 13.6x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Log reduz a assimetria e normaliza a distribuição</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>2. FAIXA_IDADE (Coluna G)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Fórmula: =SE(A2&lt;=35;"Jovem";SE(A2&lt;=50;"Adulto";SE(A2&lt;=65;"Maduro";"Senior")))</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Faixas:</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Jovem: até 35 anos</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Adulto: 36-50 anos</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Maduro: 51-65 anos</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Senior: acima de 65 anos</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>3. FAIXA_RENDA (Coluna H)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Fórmula: =SE(B2&lt;=4000;"Baixa";SE(B2&lt;=8000;"Media";SE(B2&lt;=15000;"Alta";"Muito_Alta")))</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Faixas:</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Baixa: até R$ 4.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Media: R$ 4.001 - R$ 8.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Alta: R$ 8.001 - R$ 15.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Muito_Alta: acima de R$ 15.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>4. FAIXA_VALOR (Coluna I)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Fórmula: =SE(C2&lt;=500;"Baixo";SE(C2&lt;=1500;"Medio";SE(C2&lt;=3000;"Alto";"Muito_Alto")))</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Faixas:</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Baixo: até R$ 500</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Medio: R$ 501 - R$ 1.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Alto: R$ 1.501 - R$ 3.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Muito_Alto: acima de R$ 3.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>5. RENDA_NORMALIZADA (Coluna J) - Min-Max Scaling</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Fórmula: =(B2-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Resultado: valores entre 0 e 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Útil para algoritmos sensíveis à escala (KNN, SVM, Redes Neurais)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3">
+        <f>== POR QUE CRIAR FAIXAS? ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Em árvores de decisão, variáveis numéricas geram MUITAS divisões (uma para cada valor).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Com faixas, reduzimos o número de divisões possíveis e melhoramos a interpretabilidade.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza passo 1.6 com faixas do professor
Faixas:
- Idade: Até 30, 31-50, Acima de 50
- Log Renda: Baixa (<8.5), Media (8.5-9.5), Alta (>9.5)
- Tiket Medio: Baixo (<=140), Medio (141-155), Alto (>155)
</commit_message>
<xml_diff>
--- a/dados/Dados_Tratados_Exercicios.xlsx
+++ b/dados/Dados_Tratados_Exercicios.xlsx
@@ -1995,929 +1995,457 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Idade</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Renda_Mensal</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Valor_Compras</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Numero_Compras</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Faixa de Idades</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Faixa de Log de Renda</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Faixa de tiket medio</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Classe</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Log_Renda</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Faixa_Idade</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Faixa_Renda</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Faixa_Valor</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Renda_Normalizada</t>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Particao</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2">
-        <f>'Dados Tratados'!A2</f>
+        <f>SE('Dados Tratados'!A2&lt;=30;"Até 30";SE('Dados Tratados'!A2&lt;=50;"31-50";"Acima de 50"))</f>
         <v/>
       </c>
       <c r="B2">
-        <f>'Dados Tratados'!B2</f>
+        <f>SE(LN('Dados Tratados'!B2)&lt;8,5;"Baixa";SE(LN('Dados Tratados'!B2)&lt;9,5;"Media";"Alta"))</f>
         <v/>
       </c>
       <c r="C2">
-        <f>'Dados Tratados'!C2</f>
+        <f>SE('Dados Tratados'!F2&lt;=140;"Baixo";SE('Dados Tratados'!F2&lt;=155;"Medio";"Alto"))</f>
         <v/>
       </c>
       <c r="D2">
-        <f>'Dados Tratados'!D2</f>
+        <f>'Dados Tratados'!E2</f>
         <v/>
       </c>
       <c r="E2">
-        <f>'Dados Tratados'!E2</f>
-        <v/>
-      </c>
-      <c r="F2">
-        <f>LN(B2)</f>
-        <v/>
-      </c>
-      <c r="G2">
-        <f>SE(A2&lt;=35;"Jovem";SE(A2&lt;=50;"Adulto";SE(A2&lt;=65;"Maduro";"Senior")))</f>
-        <v/>
-      </c>
-      <c r="H2">
-        <f>SE(B2&lt;=4000;"Baixa";SE(B2&lt;=8000;"Media";SE(B2&lt;=15000;"Alta";"Muito_Alta")))</f>
-        <v/>
-      </c>
-      <c r="I2">
-        <f>SE(C2&lt;=500;"Baixo";SE(C2&lt;=1500;"Medio";SE(C2&lt;=3000;"Alto";"Muito_Alto")))</f>
-        <v/>
-      </c>
-      <c r="J2">
-        <f>(B2-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <f>'Dados Tratados'!G2</f>
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <f>'Dados Tratados'!A3</f>
+        <f>SE('Dados Tratados'!A3&lt;=30;"Até 30";SE('Dados Tratados'!A3&lt;=50;"31-50";"Acima de 50"))</f>
         <v/>
       </c>
       <c r="B3">
-        <f>'Dados Tratados'!B3</f>
+        <f>SE(LN('Dados Tratados'!B3)&lt;8,5;"Baixa";SE(LN('Dados Tratados'!B3)&lt;9,5;"Media";"Alta"))</f>
         <v/>
       </c>
       <c r="C3">
-        <f>'Dados Tratados'!C3</f>
+        <f>SE('Dados Tratados'!F3&lt;=140;"Baixo";SE('Dados Tratados'!F3&lt;=155;"Medio";"Alto"))</f>
         <v/>
       </c>
       <c r="D3">
-        <f>'Dados Tratados'!D3</f>
+        <f>'Dados Tratados'!E3</f>
         <v/>
       </c>
       <c r="E3">
-        <f>'Dados Tratados'!E3</f>
-        <v/>
-      </c>
-      <c r="F3">
-        <f>LN(B3)</f>
-        <v/>
-      </c>
-      <c r="G3">
-        <f>SE(A3&lt;=35;"Jovem";SE(A3&lt;=50;"Adulto";SE(A3&lt;=65;"Maduro";"Senior")))</f>
-        <v/>
-      </c>
-      <c r="H3">
-        <f>SE(B3&lt;=4000;"Baixa";SE(B3&lt;=8000;"Media";SE(B3&lt;=15000;"Alta";"Muito_Alta")))</f>
-        <v/>
-      </c>
-      <c r="I3">
-        <f>SE(C3&lt;=500;"Baixo";SE(C3&lt;=1500;"Medio";SE(C3&lt;=3000;"Alto";"Muito_Alto")))</f>
-        <v/>
-      </c>
-      <c r="J3">
-        <f>(B3-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <f>'Dados Tratados'!G3</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <f>'Dados Tratados'!A4</f>
+        <f>SE('Dados Tratados'!A4&lt;=30;"Até 30";SE('Dados Tratados'!A4&lt;=50;"31-50";"Acima de 50"))</f>
         <v/>
       </c>
       <c r="B4">
-        <f>'Dados Tratados'!B4</f>
+        <f>SE(LN('Dados Tratados'!B4)&lt;8,5;"Baixa";SE(LN('Dados Tratados'!B4)&lt;9,5;"Media";"Alta"))</f>
         <v/>
       </c>
       <c r="C4">
-        <f>'Dados Tratados'!C4</f>
+        <f>SE('Dados Tratados'!F4&lt;=140;"Baixo";SE('Dados Tratados'!F4&lt;=155;"Medio";"Alto"))</f>
         <v/>
       </c>
       <c r="D4">
-        <f>'Dados Tratados'!D4</f>
+        <f>'Dados Tratados'!E4</f>
         <v/>
       </c>
       <c r="E4">
-        <f>'Dados Tratados'!E4</f>
-        <v/>
-      </c>
-      <c r="F4">
-        <f>LN(B4)</f>
-        <v/>
-      </c>
-      <c r="G4">
-        <f>SE(A4&lt;=35;"Jovem";SE(A4&lt;=50;"Adulto";SE(A4&lt;=65;"Maduro";"Senior")))</f>
-        <v/>
-      </c>
-      <c r="H4">
-        <f>SE(B4&lt;=4000;"Baixa";SE(B4&lt;=8000;"Media";SE(B4&lt;=15000;"Alta";"Muito_Alta")))</f>
-        <v/>
-      </c>
-      <c r="I4">
-        <f>SE(C4&lt;=500;"Baixo";SE(C4&lt;=1500;"Medio";SE(C4&lt;=3000;"Alto";"Muito_Alto")))</f>
-        <v/>
-      </c>
-      <c r="J4">
-        <f>(B4-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <f>'Dados Tratados'!G4</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <f>'Dados Tratados'!A5</f>
+        <f>SE('Dados Tratados'!A5&lt;=30;"Até 30";SE('Dados Tratados'!A5&lt;=50;"31-50";"Acima de 50"))</f>
         <v/>
       </c>
       <c r="B5">
-        <f>'Dados Tratados'!B5</f>
+        <f>SE(LN('Dados Tratados'!B5)&lt;8,5;"Baixa";SE(LN('Dados Tratados'!B5)&lt;9,5;"Media";"Alta"))</f>
         <v/>
       </c>
       <c r="C5">
-        <f>'Dados Tratados'!C5</f>
+        <f>SE('Dados Tratados'!F5&lt;=140;"Baixo";SE('Dados Tratados'!F5&lt;=155;"Medio";"Alto"))</f>
         <v/>
       </c>
       <c r="D5">
-        <f>'Dados Tratados'!D5</f>
+        <f>'Dados Tratados'!E5</f>
         <v/>
       </c>
       <c r="E5">
-        <f>'Dados Tratados'!E5</f>
-        <v/>
-      </c>
-      <c r="F5">
-        <f>LN(B5)</f>
-        <v/>
-      </c>
-      <c r="G5">
-        <f>SE(A5&lt;=35;"Jovem";SE(A5&lt;=50;"Adulto";SE(A5&lt;=65;"Maduro";"Senior")))</f>
-        <v/>
-      </c>
-      <c r="H5">
-        <f>SE(B5&lt;=4000;"Baixa";SE(B5&lt;=8000;"Media";SE(B5&lt;=15000;"Alta";"Muito_Alta")))</f>
-        <v/>
-      </c>
-      <c r="I5">
-        <f>SE(C5&lt;=500;"Baixo";SE(C5&lt;=1500;"Medio";SE(C5&lt;=3000;"Alto";"Muito_Alto")))</f>
-        <v/>
-      </c>
-      <c r="J5">
-        <f>(B5-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <f>'Dados Tratados'!G5</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <f>'Dados Tratados'!A6</f>
+        <f>SE('Dados Tratados'!A6&lt;=30;"Até 30";SE('Dados Tratados'!A6&lt;=50;"31-50";"Acima de 50"))</f>
         <v/>
       </c>
       <c r="B6">
-        <f>'Dados Tratados'!B6</f>
+        <f>SE(LN('Dados Tratados'!B6)&lt;8,5;"Baixa";SE(LN('Dados Tratados'!B6)&lt;9,5;"Media";"Alta"))</f>
         <v/>
       </c>
       <c r="C6">
-        <f>'Dados Tratados'!C6</f>
+        <f>SE('Dados Tratados'!F6&lt;=140;"Baixo";SE('Dados Tratados'!F6&lt;=155;"Medio";"Alto"))</f>
         <v/>
       </c>
       <c r="D6">
-        <f>'Dados Tratados'!D6</f>
+        <f>'Dados Tratados'!E6</f>
         <v/>
       </c>
       <c r="E6">
-        <f>'Dados Tratados'!E6</f>
-        <v/>
-      </c>
-      <c r="F6">
-        <f>LN(B6)</f>
-        <v/>
-      </c>
-      <c r="G6">
-        <f>SE(A6&lt;=35;"Jovem";SE(A6&lt;=50;"Adulto";SE(A6&lt;=65;"Maduro";"Senior")))</f>
-        <v/>
-      </c>
-      <c r="H6">
-        <f>SE(B6&lt;=4000;"Baixa";SE(B6&lt;=8000;"Media";SE(B6&lt;=15000;"Alta";"Muito_Alta")))</f>
-        <v/>
-      </c>
-      <c r="I6">
-        <f>SE(C6&lt;=500;"Baixo";SE(C6&lt;=1500;"Medio";SE(C6&lt;=3000;"Alto";"Muito_Alto")))</f>
-        <v/>
-      </c>
-      <c r="J6">
-        <f>(B6-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <f>'Dados Tratados'!G6</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <f>'Dados Tratados'!A7</f>
+        <f>SE('Dados Tratados'!A7&lt;=30;"Até 30";SE('Dados Tratados'!A7&lt;=50;"31-50";"Acima de 50"))</f>
         <v/>
       </c>
       <c r="B7">
-        <f>'Dados Tratados'!B7</f>
+        <f>SE(LN('Dados Tratados'!B7)&lt;8,5;"Baixa";SE(LN('Dados Tratados'!B7)&lt;9,5;"Media";"Alta"))</f>
         <v/>
       </c>
       <c r="C7">
-        <f>'Dados Tratados'!C7</f>
+        <f>SE('Dados Tratados'!F7&lt;=140;"Baixo";SE('Dados Tratados'!F7&lt;=155;"Medio";"Alto"))</f>
         <v/>
       </c>
       <c r="D7">
-        <f>'Dados Tratados'!D7</f>
+        <f>'Dados Tratados'!E7</f>
         <v/>
       </c>
       <c r="E7">
-        <f>'Dados Tratados'!E7</f>
-        <v/>
-      </c>
-      <c r="F7">
-        <f>LN(B7)</f>
-        <v/>
-      </c>
-      <c r="G7">
-        <f>SE(A7&lt;=35;"Jovem";SE(A7&lt;=50;"Adulto";SE(A7&lt;=65;"Maduro";"Senior")))</f>
-        <v/>
-      </c>
-      <c r="H7">
-        <f>SE(B7&lt;=4000;"Baixa";SE(B7&lt;=8000;"Media";SE(B7&lt;=15000;"Alta";"Muito_Alta")))</f>
-        <v/>
-      </c>
-      <c r="I7">
-        <f>SE(C7&lt;=500;"Baixo";SE(C7&lt;=1500;"Medio";SE(C7&lt;=3000;"Alto";"Muito_Alto")))</f>
-        <v/>
-      </c>
-      <c r="J7">
-        <f>(B7-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <f>'Dados Tratados'!G7</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <f>'Dados Tratados'!A8</f>
+        <f>SE('Dados Tratados'!A8&lt;=30;"Até 30";SE('Dados Tratados'!A8&lt;=50;"31-50";"Acima de 50"))</f>
         <v/>
       </c>
       <c r="B8">
-        <f>'Dados Tratados'!B8</f>
+        <f>SE(LN('Dados Tratados'!B8)&lt;8,5;"Baixa";SE(LN('Dados Tratados'!B8)&lt;9,5;"Media";"Alta"))</f>
         <v/>
       </c>
       <c r="C8">
-        <f>'Dados Tratados'!C8</f>
+        <f>SE('Dados Tratados'!F8&lt;=140;"Baixo";SE('Dados Tratados'!F8&lt;=155;"Medio";"Alto"))</f>
         <v/>
       </c>
       <c r="D8">
-        <f>'Dados Tratados'!D8</f>
+        <f>'Dados Tratados'!E8</f>
         <v/>
       </c>
       <c r="E8">
-        <f>'Dados Tratados'!E8</f>
-        <v/>
-      </c>
-      <c r="F8">
-        <f>LN(B8)</f>
-        <v/>
-      </c>
-      <c r="G8">
-        <f>SE(A8&lt;=35;"Jovem";SE(A8&lt;=50;"Adulto";SE(A8&lt;=65;"Maduro";"Senior")))</f>
-        <v/>
-      </c>
-      <c r="H8">
-        <f>SE(B8&lt;=4000;"Baixa";SE(B8&lt;=8000;"Media";SE(B8&lt;=15000;"Alta";"Muito_Alta")))</f>
-        <v/>
-      </c>
-      <c r="I8">
-        <f>SE(C8&lt;=500;"Baixo";SE(C8&lt;=1500;"Medio";SE(C8&lt;=3000;"Alto";"Muito_Alto")))</f>
-        <v/>
-      </c>
-      <c r="J8">
-        <f>(B8-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <f>'Dados Tratados'!G8</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <f>'Dados Tratados'!A9</f>
+        <f>SE('Dados Tratados'!A9&lt;=30;"Até 30";SE('Dados Tratados'!A9&lt;=50;"31-50";"Acima de 50"))</f>
         <v/>
       </c>
       <c r="B9">
-        <f>'Dados Tratados'!B9</f>
+        <f>SE(LN('Dados Tratados'!B9)&lt;8,5;"Baixa";SE(LN('Dados Tratados'!B9)&lt;9,5;"Media";"Alta"))</f>
         <v/>
       </c>
       <c r="C9">
-        <f>'Dados Tratados'!C9</f>
+        <f>SE('Dados Tratados'!F9&lt;=140;"Baixo";SE('Dados Tratados'!F9&lt;=155;"Medio";"Alto"))</f>
         <v/>
       </c>
       <c r="D9">
-        <f>'Dados Tratados'!D9</f>
+        <f>'Dados Tratados'!E9</f>
         <v/>
       </c>
       <c r="E9">
-        <f>'Dados Tratados'!E9</f>
-        <v/>
-      </c>
-      <c r="F9">
-        <f>LN(B9)</f>
-        <v/>
-      </c>
-      <c r="G9">
-        <f>SE(A9&lt;=35;"Jovem";SE(A9&lt;=50;"Adulto";SE(A9&lt;=65;"Maduro";"Senior")))</f>
-        <v/>
-      </c>
-      <c r="H9">
-        <f>SE(B9&lt;=4000;"Baixa";SE(B9&lt;=8000;"Media";SE(B9&lt;=15000;"Alta";"Muito_Alta")))</f>
-        <v/>
-      </c>
-      <c r="I9">
-        <f>SE(C9&lt;=500;"Baixo";SE(C9&lt;=1500;"Medio";SE(C9&lt;=3000;"Alto";"Muito_Alto")))</f>
-        <v/>
-      </c>
-      <c r="J9">
-        <f>(B9-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <f>'Dados Tratados'!G9</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <f>'Dados Tratados'!A10</f>
+        <f>SE('Dados Tratados'!A10&lt;=30;"Até 30";SE('Dados Tratados'!A10&lt;=50;"31-50";"Acima de 50"))</f>
         <v/>
       </c>
       <c r="B10">
-        <f>'Dados Tratados'!B10</f>
+        <f>SE(LN('Dados Tratados'!B10)&lt;8,5;"Baixa";SE(LN('Dados Tratados'!B10)&lt;9,5;"Media";"Alta"))</f>
         <v/>
       </c>
       <c r="C10">
-        <f>'Dados Tratados'!C10</f>
+        <f>SE('Dados Tratados'!F10&lt;=140;"Baixo";SE('Dados Tratados'!F10&lt;=155;"Medio";"Alto"))</f>
         <v/>
       </c>
       <c r="D10">
-        <f>'Dados Tratados'!D10</f>
+        <f>'Dados Tratados'!E10</f>
         <v/>
       </c>
       <c r="E10">
-        <f>'Dados Tratados'!E10</f>
-        <v/>
-      </c>
-      <c r="F10">
-        <f>LN(B10)</f>
-        <v/>
-      </c>
-      <c r="G10">
-        <f>SE(A10&lt;=35;"Jovem";SE(A10&lt;=50;"Adulto";SE(A10&lt;=65;"Maduro";"Senior")))</f>
-        <v/>
-      </c>
-      <c r="H10">
-        <f>SE(B10&lt;=4000;"Baixa";SE(B10&lt;=8000;"Media";SE(B10&lt;=15000;"Alta";"Muito_Alta")))</f>
-        <v/>
-      </c>
-      <c r="I10">
-        <f>SE(C10&lt;=500;"Baixo";SE(C10&lt;=1500;"Medio";SE(C10&lt;=3000;"Alto";"Muito_Alto")))</f>
-        <v/>
-      </c>
-      <c r="J10">
-        <f>(B10-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <f>'Dados Tratados'!G10</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <f>'Dados Tratados'!A11</f>
+        <f>SE('Dados Tratados'!A11&lt;=30;"Até 30";SE('Dados Tratados'!A11&lt;=50;"31-50";"Acima de 50"))</f>
         <v/>
       </c>
       <c r="B11">
-        <f>'Dados Tratados'!B11</f>
+        <f>SE(LN('Dados Tratados'!B11)&lt;8,5;"Baixa";SE(LN('Dados Tratados'!B11)&lt;9,5;"Media";"Alta"))</f>
         <v/>
       </c>
       <c r="C11">
-        <f>'Dados Tratados'!C11</f>
+        <f>SE('Dados Tratados'!F11&lt;=140;"Baixo";SE('Dados Tratados'!F11&lt;=155;"Medio";"Alto"))</f>
         <v/>
       </c>
       <c r="D11">
-        <f>'Dados Tratados'!D11</f>
+        <f>'Dados Tratados'!E11</f>
         <v/>
       </c>
       <c r="E11">
-        <f>'Dados Tratados'!E11</f>
-        <v/>
-      </c>
-      <c r="F11">
-        <f>LN(B11)</f>
-        <v/>
-      </c>
-      <c r="G11">
-        <f>SE(A11&lt;=35;"Jovem";SE(A11&lt;=50;"Adulto";SE(A11&lt;=65;"Maduro";"Senior")))</f>
-        <v/>
-      </c>
-      <c r="H11">
-        <f>SE(B11&lt;=4000;"Baixa";SE(B11&lt;=8000;"Media";SE(B11&lt;=15000;"Alta";"Muito_Alta")))</f>
-        <v/>
-      </c>
-      <c r="I11">
-        <f>SE(C11&lt;=500;"Baixo";SE(C11&lt;=1500;"Medio";SE(C11&lt;=3000;"Alto";"Muito_Alto")))</f>
-        <v/>
-      </c>
-      <c r="J11">
-        <f>(B11-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <f>'Dados Tratados'!G11</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12">
-        <f>'Dados Tratados'!A12</f>
+        <f>SE('Dados Tratados'!A12&lt;=30;"Até 30";SE('Dados Tratados'!A12&lt;=50;"31-50";"Acima de 50"))</f>
         <v/>
       </c>
       <c r="B12">
-        <f>'Dados Tratados'!B12</f>
+        <f>SE(LN('Dados Tratados'!B12)&lt;8,5;"Baixa";SE(LN('Dados Tratados'!B12)&lt;9,5;"Media";"Alta"))</f>
         <v/>
       </c>
       <c r="C12">
-        <f>'Dados Tratados'!C12</f>
+        <f>SE('Dados Tratados'!F12&lt;=140;"Baixo";SE('Dados Tratados'!F12&lt;=155;"Medio";"Alto"))</f>
         <v/>
       </c>
       <c r="D12">
-        <f>'Dados Tratados'!D12</f>
+        <f>'Dados Tratados'!E12</f>
         <v/>
       </c>
       <c r="E12">
-        <f>'Dados Tratados'!E12</f>
-        <v/>
-      </c>
-      <c r="F12">
-        <f>LN(B12)</f>
-        <v/>
-      </c>
-      <c r="G12">
-        <f>SE(A12&lt;=35;"Jovem";SE(A12&lt;=50;"Adulto";SE(A12&lt;=65;"Maduro";"Senior")))</f>
-        <v/>
-      </c>
-      <c r="H12">
-        <f>SE(B12&lt;=4000;"Baixa";SE(B12&lt;=8000;"Media";SE(B12&lt;=15000;"Alta";"Muito_Alta")))</f>
-        <v/>
-      </c>
-      <c r="I12">
-        <f>SE(C12&lt;=500;"Baixo";SE(C12&lt;=1500;"Medio";SE(C12&lt;=3000;"Alto";"Muito_Alto")))</f>
-        <v/>
-      </c>
-      <c r="J12">
-        <f>(B12-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <f>'Dados Tratados'!G12</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13">
-        <f>'Dados Tratados'!A13</f>
+        <f>SE('Dados Tratados'!A13&lt;=30;"Até 30";SE('Dados Tratados'!A13&lt;=50;"31-50";"Acima de 50"))</f>
         <v/>
       </c>
       <c r="B13">
-        <f>'Dados Tratados'!B13</f>
+        <f>SE(LN('Dados Tratados'!B13)&lt;8,5;"Baixa";SE(LN('Dados Tratados'!B13)&lt;9,5;"Media";"Alta"))</f>
         <v/>
       </c>
       <c r="C13">
-        <f>'Dados Tratados'!C13</f>
+        <f>SE('Dados Tratados'!F13&lt;=140;"Baixo";SE('Dados Tratados'!F13&lt;=155;"Medio";"Alto"))</f>
         <v/>
       </c>
       <c r="D13">
-        <f>'Dados Tratados'!D13</f>
+        <f>'Dados Tratados'!E13</f>
         <v/>
       </c>
       <c r="E13">
-        <f>'Dados Tratados'!E13</f>
-        <v/>
-      </c>
-      <c r="F13">
-        <f>LN(B13)</f>
-        <v/>
-      </c>
-      <c r="G13">
-        <f>SE(A13&lt;=35;"Jovem";SE(A13&lt;=50;"Adulto";SE(A13&lt;=65;"Maduro";"Senior")))</f>
-        <v/>
-      </c>
-      <c r="H13">
-        <f>SE(B13&lt;=4000;"Baixa";SE(B13&lt;=8000;"Media";SE(B13&lt;=15000;"Alta";"Muito_Alta")))</f>
-        <v/>
-      </c>
-      <c r="I13">
-        <f>SE(C13&lt;=500;"Baixo";SE(C13&lt;=1500;"Medio";SE(C13&lt;=3000;"Alto";"Muito_Alto")))</f>
-        <v/>
-      </c>
-      <c r="J13">
-        <f>(B13-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <f>'Dados Tratados'!G13</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <f>'Dados Tratados'!A14</f>
+        <f>SE('Dados Tratados'!A14&lt;=30;"Até 30";SE('Dados Tratados'!A14&lt;=50;"31-50";"Acima de 50"))</f>
         <v/>
       </c>
       <c r="B14">
-        <f>'Dados Tratados'!B14</f>
+        <f>SE(LN('Dados Tratados'!B14)&lt;8,5;"Baixa";SE(LN('Dados Tratados'!B14)&lt;9,5;"Media";"Alta"))</f>
         <v/>
       </c>
       <c r="C14">
-        <f>'Dados Tratados'!C14</f>
+        <f>SE('Dados Tratados'!F14&lt;=140;"Baixo";SE('Dados Tratados'!F14&lt;=155;"Medio";"Alto"))</f>
         <v/>
       </c>
       <c r="D14">
-        <f>'Dados Tratados'!D14</f>
+        <f>'Dados Tratados'!E14</f>
         <v/>
       </c>
       <c r="E14">
-        <f>'Dados Tratados'!E14</f>
-        <v/>
-      </c>
-      <c r="F14">
-        <f>LN(B14)</f>
-        <v/>
-      </c>
-      <c r="G14">
-        <f>SE(A14&lt;=35;"Jovem";SE(A14&lt;=50;"Adulto";SE(A14&lt;=65;"Maduro";"Senior")))</f>
-        <v/>
-      </c>
-      <c r="H14">
-        <f>SE(B14&lt;=4000;"Baixa";SE(B14&lt;=8000;"Media";SE(B14&lt;=15000;"Alta";"Muito_Alta")))</f>
-        <v/>
-      </c>
-      <c r="I14">
-        <f>SE(C14&lt;=500;"Baixo";SE(C14&lt;=1500;"Medio";SE(C14&lt;=3000;"Alto";"Muito_Alto")))</f>
-        <v/>
-      </c>
-      <c r="J14">
-        <f>(B14-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <f>'Dados Tratados'!G14</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15">
-        <f>'Dados Tratados'!A15</f>
+        <f>SE('Dados Tratados'!A15&lt;=30;"Até 30";SE('Dados Tratados'!A15&lt;=50;"31-50";"Acima de 50"))</f>
         <v/>
       </c>
       <c r="B15">
-        <f>'Dados Tratados'!B15</f>
+        <f>SE(LN('Dados Tratados'!B15)&lt;8,5;"Baixa";SE(LN('Dados Tratados'!B15)&lt;9,5;"Media";"Alta"))</f>
         <v/>
       </c>
       <c r="C15">
-        <f>'Dados Tratados'!C15</f>
+        <f>SE('Dados Tratados'!F15&lt;=140;"Baixo";SE('Dados Tratados'!F15&lt;=155;"Medio";"Alto"))</f>
         <v/>
       </c>
       <c r="D15">
-        <f>'Dados Tratados'!D15</f>
+        <f>'Dados Tratados'!E15</f>
         <v/>
       </c>
       <c r="E15">
-        <f>'Dados Tratados'!E15</f>
-        <v/>
-      </c>
-      <c r="F15">
-        <f>LN(B15)</f>
-        <v/>
-      </c>
-      <c r="G15">
-        <f>SE(A15&lt;=35;"Jovem";SE(A15&lt;=50;"Adulto";SE(A15&lt;=65;"Maduro";"Senior")))</f>
-        <v/>
-      </c>
-      <c r="H15">
-        <f>SE(B15&lt;=4000;"Baixa";SE(B15&lt;=8000;"Media";SE(B15&lt;=15000;"Alta";"Muito_Alta")))</f>
-        <v/>
-      </c>
-      <c r="I15">
-        <f>SE(C15&lt;=500;"Baixo";SE(C15&lt;=1500;"Medio";SE(C15&lt;=3000;"Alto";"Muito_Alto")))</f>
-        <v/>
-      </c>
-      <c r="J15">
-        <f>(B15-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <f>'Dados Tratados'!G15</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16">
-        <f>'Dados Tratados'!A16</f>
+        <f>SE('Dados Tratados'!A16&lt;=30;"Até 30";SE('Dados Tratados'!A16&lt;=50;"31-50";"Acima de 50"))</f>
         <v/>
       </c>
       <c r="B16">
-        <f>'Dados Tratados'!B16</f>
+        <f>SE(LN('Dados Tratados'!B16)&lt;8,5;"Baixa";SE(LN('Dados Tratados'!B16)&lt;9,5;"Media";"Alta"))</f>
         <v/>
       </c>
       <c r="C16">
-        <f>'Dados Tratados'!C16</f>
+        <f>SE('Dados Tratados'!F16&lt;=140;"Baixo";SE('Dados Tratados'!F16&lt;=155;"Medio";"Alto"))</f>
         <v/>
       </c>
       <c r="D16">
-        <f>'Dados Tratados'!D16</f>
+        <f>'Dados Tratados'!E16</f>
         <v/>
       </c>
       <c r="E16">
-        <f>'Dados Tratados'!E16</f>
-        <v/>
-      </c>
-      <c r="F16">
-        <f>LN(B16)</f>
-        <v/>
-      </c>
-      <c r="G16">
-        <f>SE(A16&lt;=35;"Jovem";SE(A16&lt;=50;"Adulto";SE(A16&lt;=65;"Maduro";"Senior")))</f>
-        <v/>
-      </c>
-      <c r="H16">
-        <f>SE(B16&lt;=4000;"Baixa";SE(B16&lt;=8000;"Media";SE(B16&lt;=15000;"Alta";"Muito_Alta")))</f>
-        <v/>
-      </c>
-      <c r="I16">
-        <f>SE(C16&lt;=500;"Baixo";SE(C16&lt;=1500;"Medio";SE(C16&lt;=3000;"Alto";"Muito_Alto")))</f>
-        <v/>
-      </c>
-      <c r="J16">
-        <f>(B16-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</f>
+        <f>'Dados Tratados'!G16</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3">
-        <f>== EXPLICAÇÃO DAS TRANSFORMAÇÕES ===</f>
+      <c r="A18" s="1">
+        <f>== FAIXAS DO PROFESSOR ===</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>1. LOG_RENDA (Coluna F)</t>
+          <t>FAIXA DE IDADES:</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Fórmula: =LN(B2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Por quê: Renda tem amplitude muito grande (2200 a 30000 = 13.6x)</t>
-        </is>
+      <c r="A21">
+        <f>SE(Idade&lt;=30;"Até 30";SE(Idade&lt;=50;"31-50";"Acima de 50"))</f>
+        <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Log reduz a assimetria e normaliza a distribuição</t>
-        </is>
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>FAIXA DE LOG DE RENDA:</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <f>SE(LN(Renda)&lt;8,5;"Baixa";SE(LN(Renda)&lt;9,5;"Media";"Alta"))</f>
+        <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>2. FAIXA_IDADE (Coluna G)</t>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Baixa: LN &lt; 8,5 (Renda &lt; ~4.900)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Fórmula: =SE(A2&lt;=35;"Jovem";SE(A2&lt;=50;"Adulto";SE(A2&lt;=65;"Maduro";"Senior")))</t>
+          <t>Media: 8,5 &lt;= LN &lt; 9,5 (Renda ~4.900 - ~13.400)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Faixas:</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Jovem: até 35 anos</t>
+          <t>Alta: LN &gt;= 9,5 (Renda &gt; ~13.400)</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Adulto: 36-50 anos</t>
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>FAIXA DE TIKET MEDIO:</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Maduro: 51-65 anos</t>
-        </is>
+      <c r="A30">
+        <f>SE(Tiket&lt;=140;"Baixo";SE(Tiket&lt;=155;"Medio";"Alto"))</f>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Senior: acima de 65 anos</t>
+          <t>Baixo: &lt;= 140</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Medio: 141-155</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="inlineStr">
-        <is>
-          <t>3. FAIXA_RENDA (Coluna H)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Fórmula: =SE(B2&lt;=4000;"Baixa";SE(B2&lt;=8000;"Media";SE(B2&lt;=15000;"Alta";"Muito_Alta")))</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Faixas:</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Baixa: até R$ 4.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Media: R$ 4.001 - R$ 8.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Alta: R$ 8.001 - R$ 15.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Muito_Alta: acima de R$ 15.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="1" t="inlineStr">
-        <is>
-          <t>4. FAIXA_VALOR (Coluna I)</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Fórmula: =SE(C2&lt;=500;"Baixo";SE(C2&lt;=1500;"Medio";SE(C2&lt;=3000;"Alto";"Muito_Alto")))</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Faixas:</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Baixo: até R$ 500</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Medio: R$ 501 - R$ 1.500</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Alto: R$ 1.501 - R$ 3.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Muito_Alto: acima de R$ 3.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="1" t="inlineStr">
-        <is>
-          <t>5. RENDA_NORMALIZADA (Coluna J) - Min-Max Scaling</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Fórmula: =(B2-MÍNIMO($B$2:$B$16))/(MÁXIMO($B$2:$B$16)-MÍNIMO($B$2:$B$16))</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Resultado: valores entre 0 e 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Útil para algoritmos sensíveis à escala (KNN, SVM, Redes Neurais)</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="3">
-        <f>== POR QUE CRIAR FAIXAS? ===</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Em árvores de decisão, variáveis numéricas geram MUITAS divisões (uma para cada valor).</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Com faixas, reduzimos o número de divisões possíveis e melhoramos a interpretabilidade.</t>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Alto: &gt; 155</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona passo 1.8 com análise ANOVA
Fórmulas:
- MÉDIASE: média por classe
- MÉDIASES: média por classe + partição
- CONT.SE/CONT.SES: contagem por critérios

Analisa poder discriminatório das variáveis
</commit_message>
<xml_diff>
--- a/dados/Dados_Tratados_Exercicios.xlsx
+++ b/dados/Dados_Tratados_Exercicios.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados Tratados" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="passo 1.5" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="passo 1.6" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="passo 1.8" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,6 +35,10 @@
     <font>
       <b val="1"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="3">
@@ -62,11 +67,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2452,4 +2458,417 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>PASSO 1.8 - PODER DISCRIMINATÓRIO DAS VARIÁVEIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Análise: As variáveis têm médias diferentes entre as classes?</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>ANÁLISE DE VARIÂNCIA (ANOVA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Variável</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Média Classe 0</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Média Classe 1</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Diferença</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Significativo?</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Idade</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>MÉDIASE('Dados Tratados'!E:E;0;'Dados Tratados'!A:A)</f>
+        <v/>
+      </c>
+      <c r="C6">
+        <f>MÉDIASE('Dados Tratados'!E:E;1;'Dados Tratados'!A:A)</f>
+        <v/>
+      </c>
+      <c r="D6">
+        <f>C6-B6</f>
+        <v/>
+      </c>
+      <c r="E6">
+        <f>SE(ABS(D6)&gt;0,2*MÉDIA(B6:C6);"SIM";"NÃO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Renda_Mensal</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>MÉDIASE('Dados Tratados'!E:E;0;'Dados Tratados'!B:B)</f>
+        <v/>
+      </c>
+      <c r="C7">
+        <f>MÉDIASE('Dados Tratados'!E:E;1;'Dados Tratados'!B:B)</f>
+        <v/>
+      </c>
+      <c r="D7">
+        <f>C7-B7</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>SE(ABS(D7)&gt;0,2*MÉDIA(B7:C7);"SIM";"NÃO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Valor_Compras</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>MÉDIASE('Dados Tratados'!E:E;0;'Dados Tratados'!C:C)</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>MÉDIASE('Dados Tratados'!E:E;1;'Dados Tratados'!C:C)</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>C8-B8</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>SE(ABS(D8)&gt;0,2*MÉDIA(B8:C8);"SIM";"NÃO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Numero_Compras</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>MÉDIASE('Dados Tratados'!E:E;0;'Dados Tratados'!D:D)</f>
+        <v/>
+      </c>
+      <c r="C9">
+        <f>MÉDIASE('Dados Tratados'!E:E;1;'Dados Tratados'!D:D)</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>C9-B9</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>SE(ABS(D9)&gt;0,2*MÉDIA(B9:C9);"SIM";"NÃO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Ticket_Medio</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>MÉDIASE('Dados Tratados'!E:E;0;'Dados Tratados'!F:F)</f>
+        <v/>
+      </c>
+      <c r="C10">
+        <f>MÉDIASE('Dados Tratados'!E:E;1;'Dados Tratados'!F:F)</f>
+        <v/>
+      </c>
+      <c r="D10">
+        <f>C10-B10</f>
+        <v/>
+      </c>
+      <c r="E10">
+        <f>SE(ABS(D10)&gt;0,2*MÉDIA(B10:C10);"SIM";"NÃO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>ANÁLISE APENAS COM DADOS DE TREINAMENTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Variável</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Média Classe 0 (Treino)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Média Classe 1 (Treino)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Diferença</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Idade</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>MÉDIASES('Dados Tratados'!A:A;'Dados Tratados'!E:E;0;'Dados Tratados'!G:G;"Treinamento")</f>
+        <v/>
+      </c>
+      <c r="C15">
+        <f>MÉDIASES('Dados Tratados'!A:A;'Dados Tratados'!E:E;1;'Dados Tratados'!G:G;"Treinamento")</f>
+        <v/>
+      </c>
+      <c r="D15">
+        <f>C15-B15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Renda_Mensal</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>MÉDIASES('Dados Tratados'!B:B;'Dados Tratados'!E:E;0;'Dados Tratados'!G:G;"Treinamento")</f>
+        <v/>
+      </c>
+      <c r="C16">
+        <f>MÉDIASES('Dados Tratados'!B:B;'Dados Tratados'!E:E;1;'Dados Tratados'!G:G;"Treinamento")</f>
+        <v/>
+      </c>
+      <c r="D16">
+        <f>C16-B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Valor_Compras</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>MÉDIASES('Dados Tratados'!C:C;'Dados Tratados'!E:E;0;'Dados Tratados'!G:G;"Treinamento")</f>
+        <v/>
+      </c>
+      <c r="C17">
+        <f>MÉDIASES('Dados Tratados'!C:C;'Dados Tratados'!E:E;1;'Dados Tratados'!G:G;"Treinamento")</f>
+        <v/>
+      </c>
+      <c r="D17">
+        <f>C17-B17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Numero_Compras</t>
+        </is>
+      </c>
+      <c r="B18">
+        <f>MÉDIASES('Dados Tratados'!D:D;'Dados Tratados'!E:E;0;'Dados Tratados'!G:G;"Treinamento")</f>
+        <v/>
+      </c>
+      <c r="C18">
+        <f>MÉDIASES('Dados Tratados'!D:D;'Dados Tratados'!E:E;1;'Dados Tratados'!G:G;"Treinamento")</f>
+        <v/>
+      </c>
+      <c r="D18">
+        <f>C18-B18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Ticket_Medio</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>MÉDIASES('Dados Tratados'!F:F;'Dados Tratados'!E:E;0;'Dados Tratados'!G:G;"Treinamento")</f>
+        <v/>
+      </c>
+      <c r="C19">
+        <f>MÉDIASES('Dados Tratados'!F:F;'Dados Tratados'!E:E;1;'Dados Tratados'!G:G;"Treinamento")</f>
+        <v/>
+      </c>
+      <c r="D19">
+        <f>C19-B19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>CONTAGEM POR CLASSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Classe 0 (Total):</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>CONT.SE('Dados Tratados'!E:E;0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Classe 1 (Total):</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>CONT.SE('Dados Tratados'!E:E;1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Classe 0 (Treino):</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>CONT.SES('Dados Tratados'!E:E;0;'Dados Tratados'!G:G;"Treinamento")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Classe 1 (Treino):</t>
+        </is>
+      </c>
+      <c r="B26">
+        <f>CONT.SES('Dados Tratados'!E:E;1;'Dados Tratados'!G:G;"Treinamento")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3">
+        <f>== INTERPRETAÇÃO ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Se a diferença entre as médias das classes for grande, a variável tem PODER DISCRIMINATÓRIO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Variáveis com médias muito diferentes entre as classes são boas para predição.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>FÓRMULAS USADAS:</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <f>MÉDIASE(intervalo_critério; critério; intervalo_média)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <f>MÉDIASES(intervalo_média; intervalo_critério1; critério1; intervalo_critério2; critério2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <f>CONT.SE(intervalo; critério)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <f>CONT.SES(intervalo1; critério1; intervalo2; critério2)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>